<commit_message>
Onboarding: find a clash-free timetable first, then improve it in the time left (the public server timed out on the Thapar sample); Thapar labs get one room each
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/colleges/thapar/thapar.xlsx
+++ b/data/colleges/thapar/thapar.xlsx
@@ -2284,7 +2284,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 1</t>
         </is>
       </c>
     </row>
@@ -2324,7 +2324,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 1</t>
         </is>
       </c>
     </row>
@@ -2364,7 +2364,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 2</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 2</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2604,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 1</t>
         </is>
       </c>
     </row>
@@ -2644,7 +2644,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 1</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2684,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 2</t>
         </is>
       </c>
     </row>
@@ -2724,7 +2724,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 2</t>
         </is>
       </c>
     </row>
@@ -2924,7 +2924,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 1</t>
         </is>
       </c>
     </row>
@@ -2964,7 +2964,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 1</t>
         </is>
       </c>
     </row>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 2</t>
         </is>
       </c>
     </row>
@@ -3044,7 +3044,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 2</t>
         </is>
       </c>
     </row>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 3</t>
         </is>
       </c>
     </row>
@@ -3252,7 +3252,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 3</t>
         </is>
       </c>
     </row>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 3</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3332,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 3</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3500,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 3</t>
         </is>
       </c>
     </row>
@@ -3540,7 +3540,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 3</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 3</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>CSED Lab 1, CSED Lab 2, CSED Lab 3</t>
+          <t>CSED Lab 3</t>
         </is>
       </c>
     </row>

</xml_diff>